<commit_message>
Add domains, ad testing, store builds, and haircuts to expense tracker
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019UN5QYknxXXe7ULkNdQNzL
</commit_message>
<xml_diff>
--- a/Subscriptions.xlsx
+++ b/Subscriptions.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -785,7 +785,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Capcut</t>
+          <t>Domains</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
@@ -793,14 +793,10 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Annual</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>14 Jun</t>
-        </is>
-      </c>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr"/>
       <c r="E10" s="9">
         <f>IF(C10="Monthly",B10,IF(C10="Annual",B10/12,0))</f>
         <v/>
@@ -809,61 +805,177 @@
         <f>IF(C10="Monthly",B10*12,IF(C10="Annual",B10,0))</f>
         <v/>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Ads - product testing</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr"/>
+      <c r="E11" s="9">
+        <f>IF(C11="Monthly",B11,IF(C11="Annual",B11/12,0))</f>
+        <v/>
+      </c>
+      <c r="F11" s="9">
+        <f>IF(C11="Monthly",B11*12,IF(C11="Annual",B11,0))</f>
+        <v/>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>Product testing ad spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>AI store making</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>180</v>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr"/>
+      <c r="E12" s="9">
+        <f>IF(C12="Monthly",B12,IF(C12="Annual",B12/12,0))</f>
+        <v/>
+      </c>
+      <c r="F12" s="9">
+        <f>IF(C12="Monthly",B12*12,IF(C12="Annual",B12,0))</f>
+        <v/>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>Shopify store builds</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Haircuts</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr"/>
+      <c r="E13" s="9">
+        <f>IF(C13="Monthly",B13,IF(C13="Annual",B13/12,0))</f>
+        <v/>
+      </c>
+      <c r="F13" s="9">
+        <f>IF(C13="Monthly",B13*12,IF(C13="Annual",B13,0))</f>
+        <v/>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>$35 x 2 per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Capcut</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>14 Jun</t>
+        </is>
+      </c>
+      <c r="E14" s="9">
+        <f>IF(C14="Monthly",B14,IF(C14="Annual",B14/12,0))</f>
+        <v/>
+      </c>
+      <c r="F14" s="9">
+        <f>IF(C14="Monthly",B14*12,IF(C14="Annual",B14,0))</f>
+        <v/>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
         <is>
           <t>Annual renewal</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="12" t="n"/>
-      <c r="C11" s="12" t="n"/>
-      <c r="D11" s="12" t="n"/>
-      <c r="E11" s="13">
-        <f>SUM(E5:E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="13">
-        <f>SUM(F5:F10)</f>
-        <v/>
-      </c>
-      <c r="G11" s="14" t="inlineStr">
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="12" t="n"/>
+      <c r="E15" s="13">
+        <f>SUM(E5:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="13">
+        <f>SUM(F5:F14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="14" t="inlineStr">
         <is>
           <t>True monthly / annual spend</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Recurring monthly cash out</t>
         </is>
       </c>
-      <c r="B13" s="16">
-        <f>SUMIF(C5:C10,"Monthly",B5:B10)</f>
-        <v/>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="B17" s="16">
+        <f>SUMIF(C5:C14,"Monthly",B5:B14)</f>
+        <v/>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>(sum of Monthly rows only)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Note's stated monthly (542)</t>
         </is>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B18" s="18" t="n">
         <v>542</v>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>excludes Zendrop</t>
         </is>

</xml_diff>

<commit_message>
Remove old 542 reference line; total includes Zendrop
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019UN5QYknxXXe7ULkNdQNzL
</commit_message>
<xml_diff>
--- a/Subscriptions.xlsx
+++ b/Subscriptions.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0.00;($#,##0.00);-"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,17 +78,6 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00777777"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00777777"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -151,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -195,12 +184,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -568,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -776,11 +759,7 @@
         <f>IF(C9="Monthly",B9*12,IF(C9="Annual",B9,0))</f>
         <v/>
       </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>Not in the '542' total on the note</t>
-        </is>
-      </c>
+      <c r="G9" s="10" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -963,21 +942,6 @@
       <c r="C17" s="10" t="inlineStr">
         <is>
           <t>(sum of Monthly rows only)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>Note's stated monthly (542)</t>
-        </is>
-      </c>
-      <c r="B18" s="18" t="n">
-        <v>542</v>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>excludes Zendrop</t>
         </is>
       </c>
     </row>

</xml_diff>